<commit_message>
Improve evaluation dashboard UI and rendering
</commit_message>
<xml_diff>
--- a/results/DAISY/DAISY_Evaluation.xlsx
+++ b/results/DAISY/DAISY_Evaluation.xlsx
@@ -488,7 +488,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="6">
@@ -528,7 +528,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -576,11 +576,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>measure_specialization</t>
+          <t>new_rule_generation</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -592,11 +592,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>capability_refinement</t>
+          <t>measure_specialization</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C3" t="n">
         <v>0</v>
@@ -608,11 +608,11 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>event_specialization</t>
+          <t>capability_refinement</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n">
         <v>0</v>
@@ -624,11 +624,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>new_rule_generation</t>
+          <t>event_specialization</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C5" t="n">
         <v>0</v>
@@ -696,7 +696,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -753,22 +753,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>situational_conflicts_1</t>
+          <t>concerns_1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>g2</t>
+          <t>g1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>measure_specialization</t>
+          <t>new_rule_generation</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="F2" t="b">
@@ -776,7 +776,8 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>r2 when MeetingUser and {patientXReligionAndComfort} then not ExaminingPatient unless {medicalEmergency}</t>
+          <t>c2 when ExamineState and ({severityOfState} &gt; StateThreshold) and PatientInCriticalCondition then not ApproachPatient
+Concern is raised</t>
         </is>
       </c>
     </row>
@@ -793,17 +794,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>g3</t>
+          <t>g2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>capability_refinement</t>
+          <t>measure_specialization</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="F3" t="b">
@@ -811,7 +812,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>r1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatientForComfortableAndAgeConsidered</t>
+          <t>r2 when MeetingUser and {patientXReligionAndComfort} then not ExaminingPatient unless {medicalEmergency}</t>
         </is>
       </c>
     </row>
@@ -828,17 +829,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>g1</t>
+          <t>g3</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>event_specialization</t>
+          <t>capability_refinement</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="F4" t="b">
@@ -846,7 +847,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Rule2 when MeetingUserWithPatientXReligion then not ExaminingPatient unless {medicalEmergency}</t>
+          <t>r1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatientForComfortableAndAgeConsidered</t>
         </is>
       </c>
     </row>
@@ -858,7 +859,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>concerns_1</t>
+          <t>situational_conflicts_1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -868,12 +869,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>new_rule_generation</t>
+          <t>event_specialization</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -881,7 +882,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination</t>
+          <t>Rule2 when MeetingUserWithPatientXReligion then not ExaminingPatient unless {medicalEmergency}</t>
         </is>
       </c>
     </row>
@@ -916,46 +917,46 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>concerns_1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>g1</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>new_rule_generation</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>r1</t>
+        </is>
+      </c>
+      <c r="F7" t="b">
+        <v>0</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
           <t>c2 when ExamineState and ({severityOfState} &gt; StateThreshold) and PatientInCriticalCondition then not ApproachPatient
 Concern is raised</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>DAISY</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>situational_conflicts_1</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>g3</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>capability_refinement</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Rule18</t>
-        </is>
-      </c>
-      <c r="F7" t="b">
-        <v>0</v>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered} and {userConsentAvalaible}) then ExaminingPatientWithConsent</t>
-        </is>
-      </c>
-    </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
@@ -969,12 +970,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>g1</t>
+          <t>g3</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>event_specialization</t>
+          <t>capability_refinement</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -987,7 +988,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Rule18 when MeetingUserWithPatientAgeUnder18 and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
+          <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered} and {userConsentAvalaible}) then ExaminingPatientWithConsent</t>
         </is>
       </c>
     </row>
@@ -1004,12 +1005,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>g2</t>
+          <t>g1</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>measure_specialization</t>
+          <t>event_specialization</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1022,7 +1023,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Rule18 when MeetingUser and ({patientComfortable} and {UserAgeUnder18}) then ExaminingPatient</t>
+          <t>Rule18 when MeetingUserWithPatientAgeUnder18 and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
     </row>
@@ -1034,22 +1035,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>conflicts_1</t>
+          <t>situational_conflicts_1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>d3</t>
+          <t>g2</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>trigger_strengthening</t>
+          <t>measure_specialization</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>Rule18</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -1057,7 +1058,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>r1 when MeetingUser and not not InformUser then InformUser</t>
+          <t>Rule18 when MeetingUser and ({patientComfortable} and {UserAgeUnder18}) then ExaminingPatient</t>
         </is>
       </c>
     </row>
@@ -1074,12 +1075,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>d4</t>
+          <t>d3</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>rule_merging</t>
+          <t>trigger_strengthening</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1092,7 +1093,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>r1 when MeetingUser then InformUser unless {not InformUser}</t>
+          <t>r1 when MeetingUser and not not InformUser then InformUser</t>
         </is>
       </c>
     </row>
@@ -1109,17 +1110,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>d2</t>
+          <t>d4</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>defeater_introduction</t>
+          <t>rule_merging</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -1127,7 +1128,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>r2 when MeetingUser then not InformUser unless {InformUser}</t>
+          <t>r1 when MeetingUser then InformUser unless {not InformUser}</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1145,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>d1</t>
+          <t>d2</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1154,7 +1155,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>r1</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -1162,7 +1163,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>r1 when MeetingUser then InformUser unless {not InformUser}</t>
+          <t>r2 when MeetingUser then not InformUser unless {InformUser}</t>
         </is>
       </c>
     </row>
@@ -1179,19 +1180,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>g2</t>
+          <t>d1</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>measure_specialization</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>defeater_introduction</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>r1</t>
+        </is>
+      </c>
       <c r="F14" t="b">
         <v>0</v>
       </c>
-      <c r="G14" t="inlineStr"/>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>r1 when MeetingUser then InformUser unless {not InformUser}</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1206,27 +1215,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>g1</t>
+          <t>g2</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>event_specialization</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>r2</t>
-        </is>
-      </c>
+          <t>measure_specialization</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="b">
         <v>0</v>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>r2 when MeetingUserInCriticalSituation then not InformUser</t>
-        </is>
-      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1236,7 +1237,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>situational_conflicts_1</t>
+          <t>conflicts_1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1251,7 +1252,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Rule18</t>
+          <t>r2</t>
         </is>
       </c>
       <c r="F16" t="b">
@@ -1259,7 +1260,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Rule18 when MeetingUserWithPatientXReligion and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
+          <t>r2 when MeetingUserInCriticalSituation then not InformUser</t>
         </is>
       </c>
     </row>
@@ -1276,12 +1277,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>g2</t>
+          <t>g1</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>measure_specialization</t>
+          <t>event_specialization</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1294,7 +1295,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeUnder18}) then ExaminingPatient</t>
+          <t>Rule18 when MeetingUserWithPatientXReligion and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
     </row>
@@ -1311,19 +1312,54 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>g2</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>measure_specialization</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Rule18</t>
+        </is>
+      </c>
+      <c r="F18" t="b">
+        <v>0</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeUnder18}) then ExaminingPatient</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>situational_conflicts_1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
           <t>g3</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>capability_refinement</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="b">
-        <v>0</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
+      <c r="E19" t="inlineStr"/>
+      <c r="F19" t="b">
+        <v>0</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1506,7 +1542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y14"/>
+  <dimension ref="A1:Y15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1671,28 +1707,28 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>situational_conflicts_1</t>
+          <t>concerns_1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>situational_conflicts</t>
+          <t>concerns</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>6</v>
       </c>
       <c r="E2" t="n">
-        <v>16.871</v>
+        <v>13.059</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>g2</t>
+          <t>g1</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>measure_specialization</t>
+          <t>new_rule_generation</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1702,525 +1738,28 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>r2</t>
+          <t>r1</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
-        <is>
-          <t>r2 when MeetingUser and {patientXReligion} then not ExaminingPatient unless {medicalEmergency}</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>r2 when MeetingUser and {patientXReligionAndComfort} then not ExaminingPatient unless {medicalEmergency}</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>The measure is specialized to include both the patient's religion and comfort level, allowing for clearer decision-making regarding examination under specific conditions.</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>def_start
-event MeetingUser
-event ExaminingPatient
-event CallHuman
-event StopSession
-measure patientComfortable:boolean
-measure patientAgeConsidered:boolean
-measure patientXReligion:boolean
-measure medicalEmergency:boolean
-measure patientXReligionAndComfort:boolean
-def_end
-rule_start
-Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
-Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
-      unless {medicalEmergency}
-Rule3 when ExaminingPatient then CallHuman
-rule_end
-concern_start
-c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
-concern_end
-purpose_start
-p1 exists ExaminingPatient
-p2 exists CallHuman
-purpose_end</t>
-        </is>
-      </c>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>1</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>2026-06-27T23:09:55.826942</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DAISY</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>situational_conflicts_1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>situational_conflicts</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E3" t="n">
-        <v>16.871</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>g3</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>capability_refinement</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>llm</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>r1</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>r1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>r1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatientForComfortableAndAgeConsidered</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>The capability ExaminingPatient is refined to specify that it applies only when the patient is comfortable and their age is considered, thus clarifying the intended behavior.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>def_start
-event MeetingUser
-event ExaminingPatient
-event CallHuman
-event StopSession
-measure patientComfortable:boolean
-measure patientAgeConsidered:boolean
-measure patientXReligion:boolean
-measure medicalEmergency:boolean
-event ExaminingPatientForComfortableAndAgeConsidered
-def_end
-rule_start
-Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
-Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
-      unless {medicalEmergency}
-Rule3 when ExaminingPatient then CallHuman
-rule_end
-concern_start
-c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
-concern_end
-purpose_start
-p1 exists ExaminingPatient
-p2 exists CallHuman
-purpose_end</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>1</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>1</v>
-      </c>
-      <c r="T3" t="n">
-        <v>1</v>
-      </c>
-      <c r="U3" t="n">
-        <v>1</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>2026-06-27T23:09:55.812954</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>DAISY</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>situational_conflicts_1</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>situational_conflicts</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E4" t="n">
-        <v>16.871</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>g1</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>event_specialization</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>llm</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>r2</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient unless {medicalEmergency}</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>Rule2 when MeetingUserWithPatientXReligion then not ExaminingPatient unless {medicalEmergency}</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>The broad event MeetingUser is specialized into a context-specific event MeetingUserWithPatientXReligion to clarify when the not ExaminingPatient rule applies.</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>def_start
-event MeetingUser
-event ExaminingPatient
-event CallHuman
-event StopSession
-measure patientComfortable:boolean
-measure patientAgeConsidered:boolean
-measure patientXReligion:boolean
-measure medicalEmergency:boolean
-event MeetingUserWithPatientXReligion
-def_end
-rule_start
-Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
-Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
-      unless {medicalEmergency}
-Rule3 when ExaminingPatient then CallHuman
-rule_end
-concern_start
-c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
-concern_end
-purpose_start
-p1 exists ExaminingPatient
-p2 exists CallHuman
-purpose_end</t>
-        </is>
-      </c>
-      <c r="N4" t="n">
-        <v>1</v>
-      </c>
-      <c r="O4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R4" t="n">
-        <v>1</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U4" t="n">
-        <v>1</v>
-      </c>
-      <c r="V4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>2026-06-27T23:09:55.795962</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>DAISY</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>concerns_1</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>concerns</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" t="n">
-        <v>21.123</v>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>g1</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>new_rule_generation</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>llm</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>r1</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
-Concern is raised</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination</t>
-        </is>
-      </c>
-      <c r="L5" t="inlineStr">
-        <is>
-          <t>A new rule is introduced to ensure that the examination only proceeds when the patient is comfortable and their age is considered, addressing the concern raised in the original rule.</t>
-        </is>
-      </c>
-      <c r="M5" t="inlineStr">
-        <is>
-          <t>def_start
-event MeetingUser
-event ExaminingPatient
-event CallHuman
-event StopSession
-measure patientComfortable:boolean
-measure patientAgeConsidered:boolean
-measure patientXReligion:boolean
-measure medicalEmergency:boolean
-def_end
-rule_start
-Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
-Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
-      unless {medicalEmergency}
-Rule3 when ExaminingPatient then CallHuman
-c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination
-rule_end
-concern_start
-c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
-concern_end
-purpose_start
-p1 exists ExaminingPatient
-p2 exists CallHuman
-purpose_end</t>
-        </is>
-      </c>
-      <c r="N5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" t="n">
-        <v>1</v>
-      </c>
-      <c r="P5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U5" t="n">
-        <v>1</v>
-      </c>
-      <c r="V5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y5" t="inlineStr">
-        <is>
-          <t>2026-06-27T23:09:09.824624</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>DAISY</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>concerns_1</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>concerns</t>
-        </is>
-      </c>
-      <c r="D6" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" t="n">
-        <v>14.338</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>g1</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>new_rule_generation</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>llm</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>r1</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
         <is>
           <t>c1 when ExamineState and ({severityOfState} &gt; StateThreshold)
 then not ApproachPatient
 Concern is raised</t>
         </is>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>c2 when ExamineState and ({severityOfState} &gt; StateThreshold) and PatientInCriticalCondition then not ApproachPatient
 Concern is raised</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
-        <is>
-          <t>A new rule is introduced to specify that if the patient is in a critical condition, the approach to the patient should be restricted to prevent further concerns.</t>
-        </is>
-      </c>
-      <c r="M6" t="inlineStr">
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>A new rule is introduced to specify that if the patient is in critical condition, the approach should be restricted to prevent potential harm.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>def_start
 event MeetingUser
@@ -2250,6 +1789,503 @@
 purpose_end</t>
         </is>
       </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:23:24.666282</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>situational_conflicts_1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>situational_conflicts</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
+        <v>16.871</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>g2</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>measure_specialization</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>llm</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>r2 when MeetingUser and {patientXReligion} then not ExaminingPatient unless {medicalEmergency}</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>r2 when MeetingUser and {patientXReligionAndComfort} then not ExaminingPatient unless {medicalEmergency}</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>The measure is specialized to include both the patient's religion and comfort level, allowing for clearer decision-making regarding examination under specific conditions.</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>def_start
+event MeetingUser
+event ExaminingPatient
+event CallHuman
+event StopSession
+measure patientComfortable:boolean
+measure patientAgeConsidered:boolean
+measure patientXReligion:boolean
+measure medicalEmergency:boolean
+measure patientXReligionAndComfort:boolean
+def_end
+rule_start
+Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
+Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
+      unless {medicalEmergency}
+Rule3 when ExaminingPatient then CallHuman
+rule_end
+concern_start
+c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
+concern_end
+purpose_start
+p1 exists ExaminingPatient
+p2 exists CallHuman
+purpose_end</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>2026-06-27T23:09:55.826942</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>situational_conflicts_1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>situational_conflicts</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" t="n">
+        <v>16.871</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>g3</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>capability_refinement</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>llm</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>r1</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>r1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>r1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatientForComfortableAndAgeConsidered</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>The capability ExaminingPatient is refined to specify that it applies only when the patient is comfortable and their age is considered, thus clarifying the intended behavior.</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>def_start
+event MeetingUser
+event ExaminingPatient
+event CallHuman
+event StopSession
+measure patientComfortable:boolean
+measure patientAgeConsidered:boolean
+measure patientXReligion:boolean
+measure medicalEmergency:boolean
+event ExaminingPatientForComfortableAndAgeConsidered
+def_end
+rule_start
+Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
+Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
+      unless {medicalEmergency}
+Rule3 when ExaminingPatient then CallHuman
+rule_end
+concern_start
+c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
+concern_end
+purpose_start
+p1 exists ExaminingPatient
+p2 exists CallHuman
+purpose_end</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>1</v>
+      </c>
+      <c r="T4" t="n">
+        <v>1</v>
+      </c>
+      <c r="U4" t="n">
+        <v>1</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>2026-06-27T23:09:55.812954</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>situational_conflicts_1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>situational_conflicts</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" t="n">
+        <v>16.871</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>g1</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>event_specialization</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>llm</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>r2</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient unless {medicalEmergency}</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Rule2 when MeetingUserWithPatientXReligion then not ExaminingPatient unless {medicalEmergency}</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>The broad event MeetingUser is specialized into a context-specific event MeetingUserWithPatientXReligion to clarify when the not ExaminingPatient rule applies.</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>def_start
+event MeetingUser
+event ExaminingPatient
+event CallHuman
+event StopSession
+measure patientComfortable:boolean
+measure patientAgeConsidered:boolean
+measure patientXReligion:boolean
+measure medicalEmergency:boolean
+event MeetingUserWithPatientXReligion
+def_end
+rule_start
+Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
+Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
+      unless {medicalEmergency}
+Rule3 when ExaminingPatient then CallHuman
+rule_end
+concern_start
+c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
+concern_end
+purpose_start
+p1 exists ExaminingPatient
+p2 exists CallHuman
+purpose_end</t>
+        </is>
+      </c>
+      <c r="N5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" t="n">
+        <v>1</v>
+      </c>
+      <c r="S5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U5" t="n">
+        <v>1</v>
+      </c>
+      <c r="V5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="inlineStr">
+        <is>
+          <t>2026-06-27T23:09:55.795962</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>concerns_1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>concerns</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" t="n">
+        <v>21.123</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>g1</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>new_rule_generation</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>llm</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>r1</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
+Concern is raised</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>A new rule is introduced to ensure that the examination only proceeds when the patient is comfortable and their age is considered, addressing the concern raised in the original rule.</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>def_start
+event MeetingUser
+event ExaminingPatient
+event CallHuman
+event StopSession
+measure patientComfortable:boolean
+measure patientAgeConsidered:boolean
+measure patientXReligion:boolean
+measure medicalEmergency:boolean
+def_end
+rule_start
+Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
+Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
+      unless {medicalEmergency}
+Rule3 when ExaminingPatient then CallHuman
+c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination
+rule_end
+concern_start
+c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
+concern_end
+purpose_start
+p1 exists ExaminingPatient
+p2 exists CallHuman
+purpose_end</t>
+        </is>
+      </c>
       <c r="N6" t="n">
         <v>0</v>
       </c>
@@ -2285,7 +2321,7 @@
       </c>
       <c r="Y6" t="inlineStr">
         <is>
-          <t>2026-06-27T15:24:05.823784</t>
+          <t>2026-06-27T23:09:09.824624</t>
         </is>
       </c>
     </row>
@@ -2297,56 +2333,185 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>situational_conflicts_1</t>
+          <t>concerns_1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>situational_conflicts</t>
+          <t>concerns</t>
         </is>
       </c>
       <c r="D7" t="n">
         <v>5</v>
       </c>
       <c r="E7" t="n">
+        <v>14.338</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>g1</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>new_rule_generation</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>llm</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>r1</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>c1 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then not ApproachPatient
+Concern is raised</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>c2 when ExamineState and ({severityOfState} &gt; StateThreshold) and PatientInCriticalCondition then not ApproachPatient
+Concern is raised</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>A new rule is introduced to specify that if the patient is in a critical condition, the approach to the patient should be restricted to prevent further concerns.</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>def_start
+event MeetingUser
+event ExamineState
+event ApproachPatient
+event CallSupport
+measure severityOfState:numeric
+measure urgentNeed:boolean
+constant StateThreshold = 100
+def_end
+rule_start
+Rule1 when MeetingUser then ExamineState
+Rule2 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then not ApproachPatient
+unless {urgentNeed}
+Rule3 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then CallSupport
+c2 when ExamineState and ({severityOfState} &gt; StateThreshold) and PatientInCriticalCondition then not ApproachPatient
+Concern is raised
+rule_end
+concern_start
+c1 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then not ApproachPatient
+concern_end
+purpose_start
+p1 exists CallSupport and {urgentNeed}
+purpose_end</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" t="n">
+        <v>0</v>
+      </c>
+      <c r="R7" t="n">
+        <v>0</v>
+      </c>
+      <c r="S7" t="n">
+        <v>0</v>
+      </c>
+      <c r="T7" t="n">
+        <v>0</v>
+      </c>
+      <c r="U7" t="n">
+        <v>1</v>
+      </c>
+      <c r="V7" t="n">
+        <v>0</v>
+      </c>
+      <c r="W7" t="n">
+        <v>0</v>
+      </c>
+      <c r="X7" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>2026-06-27T15:24:05.823784</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>situational_conflicts_1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>situational_conflicts</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" t="n">
         <v>146.131</v>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>g3</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>capability_refinement</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Rule18</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered} and {userConsentAvalaible}) then ExaminingPatientWithConsent</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>The capability ExaminingPatient is refined to specify that the examination can only proceed if user consent is available, ensuring ethical compliance.</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>def_start
 	// Events
@@ -2522,103 +2687,103 @@
 purpose_end</t>
         </is>
       </c>
-      <c r="N7" t="n">
-        <v>1</v>
-      </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" t="n">
-        <v>1</v>
-      </c>
-      <c r="T7" t="n">
-        <v>1</v>
-      </c>
-      <c r="U7" t="n">
-        <v>1</v>
-      </c>
-      <c r="V7" t="n">
-        <v>0</v>
-      </c>
-      <c r="W7" t="n">
-        <v>0</v>
-      </c>
-      <c r="X7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y7" t="inlineStr">
+      <c r="N8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" t="n">
+        <v>0</v>
+      </c>
+      <c r="S8" t="n">
+        <v>1</v>
+      </c>
+      <c r="T8" t="n">
+        <v>1</v>
+      </c>
+      <c r="U8" t="n">
+        <v>1</v>
+      </c>
+      <c r="V8" t="n">
+        <v>0</v>
+      </c>
+      <c r="W8" t="n">
+        <v>0</v>
+      </c>
+      <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="inlineStr">
         <is>
           <t>2026-06-27T12:28:21.237355</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>DAISY</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>situational_conflicts_1</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>situational_conflicts</t>
         </is>
       </c>
-      <c r="D8" t="n">
+      <c r="D9" t="n">
         <v>5</v>
       </c>
-      <c r="E8" t="n">
+      <c r="E9" t="n">
         <v>146.131</v>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>g1</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>event_specialization</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Rule18</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUserWithPatientAgeUnder18 and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>The broad event MeetingUser is specialized into a context-specific event for users under 18, allowing for clearer handling of examination rules.</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>def_start
 	// Events
@@ -2794,103 +2959,103 @@
 purpose_end</t>
         </is>
       </c>
-      <c r="N8" t="n">
-        <v>1</v>
-      </c>
-      <c r="O8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q8" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" t="n">
-        <v>1</v>
-      </c>
-      <c r="S8" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" t="n">
-        <v>0</v>
-      </c>
-      <c r="U8" t="n">
-        <v>1</v>
-      </c>
-      <c r="V8" t="n">
-        <v>0</v>
-      </c>
-      <c r="W8" t="n">
-        <v>0</v>
-      </c>
-      <c r="X8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y8" t="inlineStr">
+      <c r="N9" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" t="n">
+        <v>0</v>
+      </c>
+      <c r="T9" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>1</v>
+      </c>
+      <c r="V9" t="n">
+        <v>0</v>
+      </c>
+      <c r="W9" t="n">
+        <v>0</v>
+      </c>
+      <c r="X9" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y9" t="inlineStr">
         <is>
           <t>2026-06-27T12:28:21.221773</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>DAISY</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>situational_conflicts_1</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>situational_conflicts</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>5</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E10" t="n">
         <v>146.131</v>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>g2</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>measure_specialization</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Rule18</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {UserAgeUnder18}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>The measure of user age is specialized to specifically account for users under 18, ensuring that the examination only proceeds when appropriate for younger users.</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>def_start
 	// Events
@@ -3066,87 +3231,87 @@
 purpose_end</t>
         </is>
       </c>
-      <c r="N9" t="n">
-        <v>1</v>
-      </c>
-      <c r="O9" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q9" t="n">
-        <v>0</v>
-      </c>
-      <c r="R9" t="n">
-        <v>1</v>
-      </c>
-      <c r="S9" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" t="n">
-        <v>0</v>
-      </c>
-      <c r="U9" t="n">
-        <v>1</v>
-      </c>
-      <c r="V9" t="n">
-        <v>0</v>
-      </c>
-      <c r="W9" t="n">
-        <v>0</v>
-      </c>
-      <c r="X9" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y9" t="inlineStr">
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" t="n">
+        <v>1</v>
+      </c>
+      <c r="V10" t="n">
+        <v>0</v>
+      </c>
+      <c r="W10" t="n">
+        <v>0</v>
+      </c>
+      <c r="X10" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y10" t="inlineStr">
         <is>
           <t>2026-06-27T12:28:21.206104</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>DAISY</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>conflicts_1</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>conflicts</t>
         </is>
       </c>
-      <c r="D10" t="n">
+      <c r="D11" t="n">
         <v>5</v>
       </c>
-      <c r="E10" t="n">
+      <c r="E11" t="n">
         <v>43.072</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>g2</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G11" t="inlineStr">
         <is>
           <t>measure_specialization</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="H11" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr">
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr">
         <is>
           <t>def_start
 event MeetingUser
@@ -3158,103 +3323,103 @@
 rule_end</t>
         </is>
       </c>
-      <c r="N10" t="n">
-        <v>1</v>
-      </c>
-      <c r="O10" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" t="n">
-        <v>1</v>
-      </c>
-      <c r="S10" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" t="n">
-        <v>0</v>
-      </c>
-      <c r="U10" t="n">
-        <v>1</v>
-      </c>
-      <c r="V10" t="n">
-        <v>0</v>
-      </c>
-      <c r="W10" t="n">
-        <v>0</v>
-      </c>
-      <c r="X10" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y10" t="inlineStr">
+      <c r="N11" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1</v>
+      </c>
+      <c r="S11" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" t="n">
+        <v>1</v>
+      </c>
+      <c r="V11" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y11" t="inlineStr">
         <is>
           <t>2026-06-27T12:08:15.782579</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="12">
+      <c r="A12" t="inlineStr">
         <is>
           <t>DAISY</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>conflicts_1</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>conflicts</t>
         </is>
       </c>
-      <c r="D11" t="n">
+      <c r="D12" t="n">
         <v>5</v>
       </c>
-      <c r="E11" t="n">
+      <c r="E12" t="n">
         <v>43.072</v>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>g1</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G12" t="inlineStr">
         <is>
           <t>event_specialization</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H12" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>r2</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>r2 when MeetingUser then not InformUser</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>r2 when MeetingUserInCriticalSituation then not InformUser</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>The broad event MeetingUser is specialized into a critical situation event so the non-inform rule applies only in that context.</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>def_start
 event MeetingUser
@@ -3267,103 +3432,103 @@
 rule_end</t>
         </is>
       </c>
-      <c r="N11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" t="n">
-        <v>1</v>
-      </c>
-      <c r="S11" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" t="n">
-        <v>1</v>
-      </c>
-      <c r="V11" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y11" t="inlineStr">
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1</v>
+      </c>
+      <c r="S12" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" t="n">
+        <v>1</v>
+      </c>
+      <c r="V12" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="inlineStr">
         <is>
           <t>2026-06-27T12:08:15.762922</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>DAISY</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>situational_conflicts_1</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>situational_conflicts</t>
         </is>
       </c>
-      <c r="D12" t="n">
+      <c r="D13" t="n">
         <v>5</v>
       </c>
-      <c r="E12" t="n">
+      <c r="E13" t="n">
         <v>137.238</v>
       </c>
-      <c r="F12" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>g1</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G13" t="inlineStr">
         <is>
           <t>event_specialization</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Rule18</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUserWithPatientXReligion and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>The broad event MeetingUser is specialized into a context-specific event MeetingUserWithPatientXReligion to clarify the conditions under which ExaminingPatient applies.</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>def_start
 	// Events
@@ -3539,103 +3704,103 @@
 purpose_end</t>
         </is>
       </c>
-      <c r="N12" t="n">
-        <v>1</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" t="n">
-        <v>1</v>
-      </c>
-      <c r="S12" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" t="n">
-        <v>1</v>
-      </c>
-      <c r="V12" t="n">
-        <v>0</v>
-      </c>
-      <c r="W12" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y12" t="inlineStr">
+      <c r="N13" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" t="n">
+        <v>1</v>
+      </c>
+      <c r="V13" t="n">
+        <v>0</v>
+      </c>
+      <c r="W13" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="inlineStr">
         <is>
           <t>2026-06-27T12:03:43.612604</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+    <row r="14">
+      <c r="A14" t="inlineStr">
         <is>
           <t>DAISY</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>situational_conflicts_1</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>situational_conflicts</t>
         </is>
       </c>
-      <c r="D13" t="n">
+      <c r="D14" t="n">
         <v>5</v>
       </c>
-      <c r="E13" t="n">
+      <c r="E14" t="n">
         <v>137.238</v>
       </c>
-      <c r="F13" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>g2</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>measure_specialization</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="H14" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>Rule18</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="J14" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="K14" t="inlineStr">
         <is>
           <t>Rule18 when MeetingUser and ({patientComfortable} and {patientAgeUnder18}) then ExaminingPatient</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="L14" t="inlineStr">
         <is>
           <t>The measure UserAge is specialized to UserAgeUnder18 to ensure that the examination only occurs when the user is comfortable and under the age of 18, thus preventing conflicts with other rules regarding user consent and comfort.</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="M14" t="inlineStr">
         <is>
           <t>def_start
 	// Events
@@ -3811,87 +3976,87 @@
 purpose_end</t>
         </is>
       </c>
-      <c r="N13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="n">
-        <v>1</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" t="n">
-        <v>1</v>
-      </c>
-      <c r="V13" t="n">
-        <v>0</v>
-      </c>
-      <c r="W13" t="n">
-        <v>0</v>
-      </c>
-      <c r="X13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y13" t="inlineStr">
+      <c r="N14" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1</v>
+      </c>
+      <c r="S14" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>1</v>
+      </c>
+      <c r="V14" t="n">
+        <v>0</v>
+      </c>
+      <c r="W14" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="inlineStr">
         <is>
           <t>2026-06-27T12:03:43.596979</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
+    <row r="15">
+      <c r="A15" t="inlineStr">
         <is>
           <t>DAISY</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>situational_conflicts_1</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>situational_conflicts</t>
         </is>
       </c>
-      <c r="D14" t="n">
+      <c r="D15" t="n">
         <v>5</v>
       </c>
-      <c r="E14" t="n">
+      <c r="E15" t="n">
         <v>137.238</v>
       </c>
-      <c r="F14" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>g3</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>capability_refinement</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr">
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr">
         <is>
           <t>def_start
 	// Events
@@ -4066,40 +4231,40 @@
 purpose_end</t>
         </is>
       </c>
-      <c r="N14" t="n">
-        <v>1</v>
-      </c>
-      <c r="O14" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" t="n">
-        <v>1</v>
-      </c>
-      <c r="T14" t="n">
-        <v>1</v>
-      </c>
-      <c r="U14" t="n">
-        <v>1</v>
-      </c>
-      <c r="V14" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y14" t="inlineStr">
+      <c r="N15" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" t="n">
+        <v>0</v>
+      </c>
+      <c r="R15" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" t="n">
+        <v>1</v>
+      </c>
+      <c r="T15" t="n">
+        <v>1</v>
+      </c>
+      <c r="U15" t="n">
+        <v>1</v>
+      </c>
+      <c r="V15" t="n">
+        <v>0</v>
+      </c>
+      <c r="W15" t="n">
+        <v>0</v>
+      </c>
+      <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="inlineStr">
         <is>
           <t>2026-06-27T12:03:43.583773</t>
         </is>
@@ -4281,56 +4446,185 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>situational_conflicts_1</t>
+          <t>concerns_1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>situational_conflicts</t>
+          <t>concerns</t>
         </is>
       </c>
       <c r="D2" t="n">
         <v>6</v>
       </c>
       <c r="E2" t="n">
+        <v>13.059</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>g1</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>new_rule_generation</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>llm</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>r1</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>c1 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then not ApproachPatient
+Concern is raised</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>c2 when ExamineState and ({severityOfState} &gt; StateThreshold) and PatientInCriticalCondition then not ApproachPatient
+Concern is raised</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>A new rule is introduced to specify that if the patient is in critical condition, the approach should be restricted to prevent potential harm.</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>def_start
+event MeetingUser
+event ExamineState
+event ApproachPatient
+event CallSupport
+measure severityOfState:numeric
+measure urgentNeed:boolean
+constant StateThreshold = 100
+def_end
+rule_start
+Rule1 when MeetingUser then ExamineState
+Rule2 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then not ApproachPatient
+unless {urgentNeed}
+Rule3 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then CallSupport
+c2 when ExamineState and ({severityOfState} &gt; StateThreshold) and PatientInCriticalCondition then not ApproachPatient
+Concern is raised
+rule_end
+concern_start
+c1 when ExamineState and ({severityOfState} &gt; StateThreshold)
+then not ApproachPatient
+concern_end
+purpose_start
+p1 exists CallSupport and {urgentNeed}
+purpose_end</t>
+        </is>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U2" t="n">
+        <v>1</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>2026-06-28T01:23:24.666282</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DAISY</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>situational_conflicts_1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>situational_conflicts</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" t="n">
         <v>16.871</v>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>g2</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>measure_specialization</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>llm</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>r2</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>r2 when MeetingUser and {patientXReligion} then not ExaminingPatient unless {medicalEmergency}</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>r2 when MeetingUser and {patientXReligionAndComfort} then not ExaminingPatient unless {medicalEmergency}</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>The measure is specialized to include both the patient's religion and comfort level, allowing for clearer decision-making regarding examination under specific conditions.</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>def_start
 event MeetingUser
@@ -4358,167 +4652,42 @@
 purpose_end</t>
         </is>
       </c>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U2" t="n">
-        <v>1</v>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="n">
-        <v>0</v>
-      </c>
-      <c r="X2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y2" t="inlineStr">
+      <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>1</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>1</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
         <is>
           <t>2026-06-27T23:09:55.826942</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>DAISY</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>concerns_1</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>concerns</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E3" t="n">
-        <v>21.123</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>g1</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>new_rule_generation</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>llm</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>r1</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
-Concern is raised</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>A new rule is introduced to ensure that the examination only proceeds when the patient is comfortable and their age is considered, addressing the concern raised in the original rule.</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>def_start
-event MeetingUser
-event ExaminingPatient
-event CallHuman
-event StopSession
-measure patientComfortable:boolean
-measure patientAgeConsidered:boolean
-measure patientXReligion:boolean
-measure medicalEmergency:boolean
-def_end
-rule_start
-Rule1 when MeetingUser and ({patientComfortable} and {patientAgeConsidered}) then ExaminingPatient
-Rule2 when MeetingUser and {patientXReligion} then not ExaminingPatient
-      unless {medicalEmergency}
-Rule3 when ExaminingPatient then CallHuman
-c2 when MeetingUser and {patientComfortable} and {patientAgeConsidered} then ProceedWithExamination
-rule_end
-concern_start
-c1 when MeetingUser and ((not {patientComfortable}) or (not {patientAgeConsidered})) then ExaminingPatient
-concern_end
-purpose_start
-p1 exists ExaminingPatient
-p2 exists CallHuman
-purpose_end</t>
-        </is>
-      </c>
-      <c r="N3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" t="n">
-        <v>1</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U3" t="n">
-        <v>1</v>
-      </c>
-      <c r="V3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0</v>
-      </c>
-      <c r="X3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>2026-06-27T23:09:09.824624</t>
         </is>
       </c>
     </row>

</xml_diff>